<commit_message>
Anomalies SF1-RPS3 — 18/09/2026
</commit_message>
<xml_diff>
--- a/presentation/SF1-RPS3/anomalies.xlsx
+++ b/presentation/SF1-RPS3/anomalies.xlsx
@@ -21,13 +21,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -48,7 +51,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -56,13 +59,19 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -431,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:U37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -566,36 +575,36 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>12320491</v>
+        <v>10163533</v>
       </c>
       <c r="B2" t="n">
-        <v>4002310385</v>
+        <v>4202859</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>remise en état niveau radar du bac d'aci</t>
+          <t>Controle analyseur</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>OR004002310385</t>
+          <t>OR000004202859</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-LIMBAT-0T7402</t>
+          <t>SF01-PS-PS03-SECEAU-0T7101-CSUR-AI2508</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>BAC DE STOCKAGE ACIDE SULFURIQUE T5401B</t>
+          <t>ANALYSEUR DE CONDUCTIVITE RET CONDENSATS</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>S-PC-T5401B</t>
+          <t>S-PC-AI2508</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -605,7 +614,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>GM4</t>
+          <t>GM0</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -615,7 +624,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>LANC CCRP PART RIMP</t>
+          <t>BLOQ CLOT CCRP NEFF PART</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -625,14 +634,14 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>BENMOUSSA1</t>
+          <t>HMIDOUCH</t>
         </is>
       </c>
       <c r="P2" s="2" t="n">
-        <v>46230</v>
+        <v>45721</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>46217</v>
+        <v>45714</v>
       </c>
       <c r="R2" t="n">
         <v>1</v>
@@ -644,30 +653,30 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12576342</v>
+        <v>13503107</v>
       </c>
       <c r="B3" t="n">
-        <v>4002310386</v>
+        <v>4002621692</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>contrôle film gard du refroidisseur de p</t>
+          <t>Calibrage des pH-mètres d'eau de mer</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>OR004002310386</t>
+          <t>OR004002621692</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -718,62 +727,62 @@
         </is>
       </c>
       <c r="P3" s="2" t="n">
-        <v>46230</v>
+        <v>46273</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>46217</v>
+        <v>46267</v>
       </c>
       <c r="R3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>12634921</v>
+        <v>13505896</v>
       </c>
       <c r="B4" t="n">
-        <v>4002310387</v>
+        <v>4002621694</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>contrôle film Gard de production ps3</t>
+          <t>Etalonnage de PIC1420</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>OR004002310387</t>
+          <t>OR004002621694</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-SECACI-0E7302</t>
+          <t>SF01-PS-PS03-SECSSL-0T7307-CSUR-PI1420</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>REFROIDISSEUR D'ACIDE PRODUCTION PSIII</t>
+          <t>TRANSMETTEUR DE PRESSION DE VAPEUR MP</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>S-PC-E7302</t>
+          <t>S-PC-PI1420</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -783,7 +792,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>GM4</t>
+          <t>GM0</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -807,62 +816,62 @@
         </is>
       </c>
       <c r="P4" s="2" t="n">
-        <v>46230</v>
+        <v>46274</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>46217</v>
+        <v>46267</v>
       </c>
       <c r="R4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>12718433</v>
+        <v>13521059</v>
       </c>
       <c r="B5" t="n">
-        <v>4002310388</v>
+        <v>4002621695</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>aménagement chemein de cable coté HRS</t>
+          <t>remise en état de TI1400 et TI1436A</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>OR004002310388</t>
+          <t>OR004002621695</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-SECACI-0C7303</t>
+          <t>SF01-PS-PS03-SECSSL-0T7202</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>TOUR D'ACIDE HRS PSIII</t>
+          <t>BAC A SOUFRE T7202 ATELIER PSIII</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>S-PC-C7303</t>
+          <t>S-PC-T7202</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -872,7 +881,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>GM4</t>
+          <t>GM7</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -896,62 +905,62 @@
         </is>
       </c>
       <c r="P5" s="2" t="n">
-        <v>46231</v>
+        <v>46274</v>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>46217</v>
+        <v>46267</v>
       </c>
       <c r="R5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>12781842</v>
+        <v>13521092</v>
       </c>
       <c r="B6" t="n">
-        <v>4002310389</v>
+        <v>4002621696</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>changement arrêt d'urgence local de la t</t>
+          <t>changement du manomètre entrée filtre d'</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>OR004002310389</t>
+          <t>OR004002621696</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-SECAIR-0K7301</t>
+          <t>SF01-PS-PS03-SECEMR-S7306B</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TURBOSOUFFLANTE PSIII</t>
+          <t>FILTRE A EAU DE MER S7306B PSIII</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>S-PC-K7301</t>
+          <t>S-PC-S7306B</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -985,62 +994,62 @@
         </is>
       </c>
       <c r="P6" s="2" t="n">
-        <v>46217</v>
+        <v>46272</v>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>46217</v>
+        <v>46267</v>
       </c>
       <c r="R6" t="n">
         <v>2</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution 1mois&lt; &lt;3mois</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs. | Reduire les OT en execution entre 1 et 3 mois.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>12814868</v>
+        <v>13521184</v>
       </c>
       <c r="B7" t="n">
-        <v>4002310390</v>
+        <v>4002621697</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Contrôle de la vanne de désurchauffe TV2</t>
+          <t>calibrage du débitmètre d'acide de produ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>OR004002310390</t>
+          <t>OR004002621697</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SF01</t>
+          <t>SF01-PS-PS03-SECACI-0D7303-CSUR-FI1300</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>DIVISION MAROC CHIMIE</t>
+          <t>DEBITMETRE ELECTROMAGNTIQUE ACID PRODUIT</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>NOUVEAU PT_SAP</t>
+          <t>S-PC-FI1300</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1050,7 +1059,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>GM1</t>
+          <t>GM0</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1074,62 +1083,62 @@
         </is>
       </c>
       <c r="P7" s="2" t="n">
-        <v>46231</v>
+        <v>46274</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>46217</v>
+        <v>46267</v>
       </c>
       <c r="R7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>12855071</v>
+        <v>13535996</v>
       </c>
       <c r="B8" t="n">
-        <v>4002310391</v>
+        <v>4002698049</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>remise en état FI1430</t>
+          <t>Remise en état transmetteur de pression</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>OR004002310391</t>
+          <t>OR004002698049</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-LIMBAT-SOUFRE</t>
+          <t>SF01-PS-PS03-SECEMR-S7306A</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>CIRCUIT SOUFRE LIMITE BATTERIE PSIII</t>
+          <t>FILTRE A EAU DE MER S7306A PSIII</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>S-PC-PSIII-SOUFRE</t>
+          <t>S-PC-S7306A</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1139,7 +1148,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>GM4</t>
+          <t>GM0</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1163,62 +1172,62 @@
         </is>
       </c>
       <c r="P8" s="2" t="n">
-        <v>46231</v>
+        <v>46273</v>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>46217</v>
+        <v>46272</v>
       </c>
       <c r="R8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>12955192</v>
+        <v>13537253</v>
       </c>
       <c r="B9" t="n">
-        <v>4002310468</v>
+        <v>4002698051</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Remise en état de l'analyseur AI1001</t>
+          <t>étanchement fuite d'acide sur presse éto</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>OR004002310468</t>
+          <t>OR004002698051</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-SECACI-AI1001</t>
+          <t>SF01-PS-PS03-SECACI-0D7303-CSUR-LV1200</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ANALYSEUR DE GAZ SO2/O2</t>
+          <t>VANNE DE REG DE NIVEAU BAC DE ROULEMENT</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>S-PC-AI1001/1002</t>
+          <t>S-PC-LV1200</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1252,62 +1261,62 @@
         </is>
       </c>
       <c r="P9" s="2" t="n">
-        <v>46224</v>
+        <v>46273</v>
       </c>
       <c r="Q9" s="2" t="n">
-        <v>46217</v>
+        <v>46272</v>
       </c>
       <c r="R9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>12962167</v>
+        <v>13537258</v>
       </c>
       <c r="B10" t="n">
-        <v>4002310469</v>
+        <v>4002698052</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Etalonnage du débitmètre FI3110</t>
+          <t>étanchement de fuite d'acide sur circuit</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>OR004002310469</t>
+          <t>OR004002698052</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-SECVAP-0D7302-CSUR-FI3110</t>
+          <t>SF01-PS-PS03-SECACI-0E7301</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>DEBITMETRE VAPEUR MP S/BALLON CHAUD HRS</t>
+          <t>REFROIDISSEUR D'ACIDE DE SECHAGE PSIII</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>S-PC-FI3110</t>
+          <t>S-PC-E7301</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1317,7 +1326,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>GM0</t>
+          <t>GM4</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1341,55 +1350,55 @@
         </is>
       </c>
       <c r="P10" s="2" t="n">
-        <v>46225</v>
+        <v>46272</v>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>46217</v>
+        <v>46272</v>
       </c>
       <c r="R10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>13139773</v>
+        <v>13537345</v>
       </c>
       <c r="B11" t="n">
-        <v>4002310471</v>
+        <v>4002698054</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Etanchement fuite de soufre sur débitmèt</t>
+          <t>démontage et remontage du manomètre refr</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>OR004002310471</t>
+          <t>OR004002698054</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-SECSAS-CIRACS-CSUR</t>
+          <t>SF01-PS-PS03-SECACI-0E7301-CANA</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>CONTROLE ET SURVEILLANCE</t>
+          <t>ACCESSOIR REFROIDISSEUR SECHANTE PSIII</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1402,7 +1411,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>GM0</t>
+          <t>GM4</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1426,64 +1435,60 @@
         </is>
       </c>
       <c r="P11" s="2" t="n">
-        <v>46226</v>
+        <v>46272</v>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>46217</v>
+        <v>46272</v>
       </c>
       <c r="R11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>12919497</v>
+        <v>13579511</v>
       </c>
       <c r="B12" t="n">
-        <v>4002310474</v>
+        <v>4002698055</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Remise en état de AI2509</t>
+          <t>contrôle et remise en état du film gard</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>OR004002310474</t>
+          <t>OR004002698055</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-SECEAU-0T7101-CSUR-AI2509</t>
+          <t>SF01-PS-PS03-SECACI-0E7302-CANA-ELECTROD</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ANALYSEUR DE CONDUCTIVITE RET CONDENSATS</t>
+          <t>ELCTRODES REFROIDIS E7302 PSIII</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>S-PC-AI2509</t>
-        </is>
-      </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>SF1-RPS3</t>
@@ -1491,7 +1496,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>GM0</t>
+          <t>GM4</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1515,64 +1520,60 @@
         </is>
       </c>
       <c r="P12" s="2" t="n">
-        <v>46246</v>
+        <v>46272</v>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>46217</v>
+        <v>46272</v>
       </c>
       <c r="R12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12930821</v>
+        <v>13536110</v>
       </c>
       <c r="B13" t="n">
-        <v>4002310475</v>
+        <v>4002698165</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Remise en état de TI1150</t>
+          <t>Installation manomètre et thermomètre</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>OR004002310475</t>
+          <t>OR004002698165</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-SECAIR-0C7301-CSUR-TI1150</t>
+          <t>SF01-PS-PS03-SECACI-0E7302-CSUR</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SONDE DE TEMP ACIDE VERS 2EME ETAGE HRS</t>
+          <t>CONTROLE ET SURVEILLANCE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>S-PC-TI1150</t>
-        </is>
-      </c>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>SF1-RPS3</t>
@@ -1604,60 +1605,64 @@
         </is>
       </c>
       <c r="P13" s="2" t="n">
-        <v>46246</v>
+        <v>46272</v>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>46217</v>
+        <v>46272</v>
       </c>
       <c r="R13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>13056329</v>
+        <v>13612824</v>
       </c>
       <c r="B14" t="n">
-        <v>4002317970</v>
+        <v>4002711997</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>controle thermomètre d'eau filtrée ent</t>
+          <t>calibrage analyseur de gaz</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>OR004002317970</t>
+          <t>OR004002711997</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-LIMBAT-EAUFIL-CSUR</t>
+          <t>SF01-PS-PS03-SECACI-AI1001</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>CONTROLE ET SURVEILLANCE</t>
+          <t>ANALYSEUR DE GAZ SO2/O2</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>S-PC-AI1001/1002</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr">
         <is>
           <t>SF1-RPS3</t>
@@ -1685,64 +1690,66 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>BENMOUSSA1</t>
+          <t>MOUSSAHIF</t>
         </is>
       </c>
       <c r="P14" s="2" t="n">
-        <v>46225</v>
+        <v>46279</v>
       </c>
       <c r="Q14" s="2" t="n">
-        <v>46219</v>
+        <v>46274</v>
       </c>
       <c r="R14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" t="n">
+        <v>13607838</v>
+      </c>
       <c r="B15" t="n">
-        <v>4002462900</v>
+        <v>4002723015</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Changement des TRANSMETTEUR  PH-METRE 10</t>
+          <t>changement du thermocouple TI1005B</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>OR004002462900</t>
+          <t>OR004002723015</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-SECACI-0E7301-CSUR-AI3301</t>
+          <t>SF01-PS-PS03-SECGAZ-0F7301-CSUR-TI1005B</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ANALYSEUR PH EAU DE MER REFROID SECHAGE</t>
+          <t>THERMOCOUPLE GAZ SORTIE FOUR</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>S-PC-AI3301</t>
+          <t>S-PC-TI1005B</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1762,7 +1769,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>LANC ARCO CCRP ERCT RIMP</t>
+          <t>LANC CCRP PART RIMP</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1772,64 +1779,66 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>FATHELLAH</t>
+          <t>BENMOUSSA1</t>
         </is>
       </c>
       <c r="P15" s="2" t="n">
-        <v>46238</v>
+        <v>46280</v>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>46238</v>
+        <v>46276</v>
       </c>
       <c r="R15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="n">
+        <v>13624036</v>
+      </c>
       <c r="B16" t="n">
-        <v>4002462901</v>
+        <v>4002723016</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Changement des SONDE DE CONCENTRATION 22</t>
+          <t>Contrôle et remise en état du niveau rad</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>OR004002462901</t>
+          <t>OR004002723016</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-SECACI-AI1001</t>
+          <t>SF01-PS-PS03-SECSAS-0T7402-CSUR-LI1302</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>ANALYSEUR DE GAZ SO2/O2</t>
+          <t>TRANSMETTEUR DE NIVEAU RADAR BAC T7402</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>S-PC-AI1001/1002</t>
+          <t>S-PC-LI1302</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1849,7 +1858,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>LANC ARCO CCRP ERCT MMEf RIMP</t>
+          <t>LANC CCRP PART RIMP</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1859,66 +1868,66 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>FATHELLAH</t>
+          <t>BENMOUSSA1</t>
         </is>
       </c>
       <c r="P16" s="2" t="n">
-        <v>46238</v>
+        <v>46280</v>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>46238</v>
+        <v>46276</v>
       </c>
       <c r="R16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Chef d'atelier</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>10163533</v>
+        <v>13628499</v>
       </c>
       <c r="B17" t="n">
-        <v>4202859</v>
+        <v>4002723017</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Controle analyseur</t>
+          <t>étalonnage et calibrage de l'analyseur d</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>OR000004202859</t>
+          <t>OR004002723017</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-SECEAU-0T7101-CSUR-AI2508</t>
+          <t>SF01-PS-PS03-SECACI-AI1001</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ANALYSEUR DE CONDUCTIVITE RET CONDENSATS</t>
+          <t>ANALYSEUR DE GAZ SO2/O2</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>S-PC-AI2508</t>
+          <t>S-PC-AI1001/1002</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1938,7 +1947,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>CLOT CCRP NEFF PART</t>
+          <t>LANC CCRP PART RIMP</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1948,64 +1957,66 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>HMIDOUCH</t>
+          <t>BENMOUSSA1</t>
         </is>
       </c>
       <c r="P17" s="2" t="n">
-        <v>45721</v>
+        <v>46281</v>
       </c>
       <c r="Q17" s="2" t="n">
-        <v>45714</v>
+        <v>46276</v>
       </c>
       <c r="R17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>OT CONFIME</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Agent de saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>Confirmer les OT termines (statut CONF).</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="n">
+        <v>13677188</v>
+      </c>
       <c r="B18" t="n">
-        <v>4001062342</v>
+        <v>4002761934</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Démontage et remontage aprés controle</t>
+          <t>controle de la vanne TV1105</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>OR004001062342</t>
+          <t>OR004002761934</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-SECGAZ-0F7301-CSUR-HV1005</t>
+          <t>SF01-PS-PS03-SECAIR-0C7301-CSUR-TV1105</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SERVOMOTEUR ELECTRIQUE BY-PASS GAZ CHAUD</t>
+          <t>VANNE DE REG DE TEMP D'ACIDE E/T.SECHAGE</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>S-PC-HV1005</t>
+          <t>S-PC-TV1105</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2025,7 +2036,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>TCLO CNFP CCRP ERCT JBFI PART RIMP</t>
+          <t>LANC ARCO CCRP MMEf RIMP</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2035,66 +2046,66 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>BENMOUSSA1</t>
+          <t>MOUSSAHIF</t>
         </is>
       </c>
       <c r="P18" s="2" t="n">
-        <v>46035</v>
+        <v>46281</v>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>46035</v>
+        <v>46280</v>
       </c>
       <c r="R18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>OT CONFIME</t>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Agent de saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Confirmer les OT termines (statut CONF).</t>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>10148432</v>
+        <v>13668429</v>
       </c>
       <c r="B19" t="n">
-        <v>4206511</v>
+        <v>4002761983</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>mise en service analyseur taux de cendre</t>
+          <t>élimination alarme us1005 au niveau de l</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>OR000004206511</t>
+          <t>OR004002761983</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SF01-PS-PS03-STINST-000DCS</t>
+          <t>SF01-PS-PS03-SECAIR-0K7301</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>SYSTEME NUMERIQUE DE CONCTROLE COMMANDE</t>
+          <t>TURBOSOUFFLANTE PSIII</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>S-PC-PSIII-DCS</t>
+          <t>S-PC-K7301</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2104,51 +2115,1619 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>MOUSSAHIF</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="Q19" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="R19" t="n">
+        <v>2</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Augmenter le taux de réalisation et clôturer techniquement les OT terminés (CLOT/TCLO). | Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>13677189</v>
+      </c>
+      <c r="B20" t="n">
+        <v>4002761939</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>remise en état LI1434</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>OR004002761939</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECSSL-0T7202-CSUR-LI1434</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>TRANSMETTEUR DE NIVEAU RADAR BAC T7202</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>S-PC-LI1434</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
           <t>GM0</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>SF01</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>MOUSSAHIF</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="Q20" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="R20" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>13668427</v>
+      </c>
+      <c r="B21" t="n">
+        <v>4002761982</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>étalonnage des niveaux radars des bacs d</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>OR004002761982</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECSAS-0T7401</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>BAC DE STOCKAGE ACIDE SULFURIQUE T7401</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>S-PC-T7401</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>MOUSSAHIF</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="Q21" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>13638540</v>
+      </c>
+      <c r="B22" t="n">
+        <v>4002762394</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CONTROLE  DETECTEUR NIVEAU</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>OR004002762394</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECVAP-0D7301-CSUR-LE2210</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>DETECTEUR DE NIVEAU ELECTR CHAUDIERE HP</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>S-PC-LE2210</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>GM0</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>MOUSSAHIF</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="Q22" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="R22" t="n">
+        <v>1</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>13638531</v>
+      </c>
+      <c r="B23" t="n">
+        <v>4002762395</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CONTROLE INSTR P7103A</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>OR004002762395</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECEAU-P7103A-CSUR-ACCINSTR</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>ACCESSOIRES INSTRUMENTATION PPE P7103A</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>GM0</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>MOUSSAHIF</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="Q23" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="R23" t="n">
+        <v>1</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>13638524</v>
+      </c>
+      <c r="B24" t="n">
+        <v>4002762464</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CONTROLE MANOMETRE</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>OR004002762464</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECACI-0E7301-CSUR-PI1101</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>MANOMETRE ACIDE E/REFROIDISSEUR SECHAGE</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>S-PC-PI1101</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>GM0</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>MOUSSAHIF</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="Q24" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="R24" t="n">
+        <v>1</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>13637419</v>
+      </c>
+      <c r="B25" t="n">
+        <v>4002762610</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CONTROLE DETECTEUR NIVEAU</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>OR004002762610</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECEAU-0T7102-CSUR-LSHH2548</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>DETECTEUR DE NIVEAU MAGNETIQUE BACH ALIM</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>GM0</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>MOUSSAHIF</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="Q25" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="R25" t="n">
+        <v>1</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>10478553</v>
+      </c>
+      <c r="B26" t="n">
+        <v>4550860</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>remise en état PI1923</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>OR000004550860</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECAIR</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>SECTION AIR COMBUSTION DATELIER PSIII</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>GM0</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
         <is>
           <t>TCLO CONF CCRP JBFI PART RIMP</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>SOPL</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>MATAR1</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="n">
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>JALLOU</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="n">
         <v>45836</v>
       </c>
-      <c r="Q19" s="2" t="n">
-        <v>45716</v>
-      </c>
-      <c r="R19" t="n">
+      <c r="Q26" s="2" t="n">
+        <v>45793</v>
+      </c>
+      <c r="R26" t="n">
         <v>1</v>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="S26" t="inlineStr">
         <is>
           <t>OT_COR_EGAL</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>Agent de saisie</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>Verifier l imputation des couts reels des OT correctifs.</t>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>11752227</v>
+      </c>
+      <c r="B27" t="n">
+        <v>4000986923</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>étalonnage du niveau LI1302</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>OR004000986923</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECSAS-0T7402-CSUR-LI1302</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>TRANSMETTEUR DE NIVEAU RADAR BAC T7402</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>S-PC-LI1302</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>GM0</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>JALLOU</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="n">
+        <v>46016</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>46021</v>
+      </c>
+      <c r="R27" t="n">
+        <v>1</v>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>11784232</v>
+      </c>
+      <c r="B28" t="n">
+        <v>4000986924</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>aménagement des cables au stockage acide</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>OR004000986924</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECSAS</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>STOCKAGE ACIDE SULFURIQUE ATELIER PSIII</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>SA-PC-PSIII-SSU</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>JALLOU</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="n">
+        <v>46016</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>46021</v>
+      </c>
+      <c r="R28" t="n">
+        <v>1</v>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>11849444</v>
+      </c>
+      <c r="B29" t="n">
+        <v>4001005126</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>remise en état du OS N°2</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>OR004001005126</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-STINST-000DCS-ARPC-POSTOS02</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>POSTE OPERATEUR OS02</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>GM0</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>JALLOU</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="n">
+        <v>46023</v>
+      </c>
+      <c r="Q29" s="2" t="n">
+        <v>46023</v>
+      </c>
+      <c r="R29" t="n">
+        <v>1</v>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="n">
+        <v>4001079413</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Changement de la sonde de concentration</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>OR004001079413</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECACI-0C7303-CSUR-AI3000A</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>ANALYSEUR DE CONDUCTIVITE D'ACIDE S/HRS</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>S-PC-AI3000A</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>GM0</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>BENMOUSSA1</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="n">
+        <v>46041</v>
+      </c>
+      <c r="Q30" s="2" t="n">
+        <v>46041</v>
+      </c>
+      <c r="R30" t="n">
+        <v>1</v>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="n">
+        <v>4001080474</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Installation des transmetteurs de perte</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>OR004001080474</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-COMMUN-INSTRU-CSUR</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>CONTROLE ET SURVEILLANCE</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>GM0</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>BENMOUSSA1</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>46048</v>
+      </c>
+      <c r="Q31" s="2" t="n">
+        <v>46042</v>
+      </c>
+      <c r="R31" t="n">
+        <v>1</v>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="n">
+        <v>4001081620</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Contrôle de la vanne de régulation</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>OR004001081620</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECSSL-0T7307-CSUR-PV1420</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>VANNE DE REG DE PRESSION VAPEUR</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>S-PC-PV1420</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>GM0</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>BENMOUSSA1</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="n">
+        <v>46052</v>
+      </c>
+      <c r="Q32" s="2" t="n">
+        <v>46042</v>
+      </c>
+      <c r="R32" t="n">
+        <v>1</v>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="n">
+        <v>4001081701</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Contrôle de la vanne de régulation</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>OR004001081701</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECEAU-0T7102-CSUR-LV2547</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>VANNE DE REG DE NIVEAU BACHE ALIMENTAIRE</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>S-PC-LV2547</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>GM0</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>BENMOUSSA1</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="n">
+        <v>46042</v>
+      </c>
+      <c r="Q33" s="2" t="n">
+        <v>46042</v>
+      </c>
+      <c r="R33" t="n">
+        <v>1</v>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="n">
+        <v>4001084025</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Contrôle et entretien de la vanne HV2206</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>OR004001084025</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECGAZ-0E7304-CSUR-HV2206</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>VANNE DE REG VAPEUR HP S/SURCH 1B</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>S-PC-HV2206</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>GM0</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>BENMOUSSA1</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="n">
+        <v>46060</v>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>46042</v>
+      </c>
+      <c r="R34" t="n">
+        <v>1</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="n">
+        <v>4001084026</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>REVISION VANNE TV2207</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>OR004001084026</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECGAZ-SEC4AC-CSUR-TV2207</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>VANNE DE REG TEMPERATURE VAP HP S/ 1B</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>S-PC-TV2207</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>GM0</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>BENMOUSSA1</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="n">
+        <v>46060</v>
+      </c>
+      <c r="Q35" s="2" t="n">
+        <v>46042</v>
+      </c>
+      <c r="R35" t="n">
+        <v>1</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="n">
+        <v>4001084027</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>REVISION VANNE PV2250</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>OR004001084027</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECVAP-COMMUN-CSUR-PV2250</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>VANNE DE REG DE PRESSION VAPEUR HP</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>S-PC-PV2250</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>GM0</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>BENMOUSSA1</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="n">
+        <v>46052</v>
+      </c>
+      <c r="Q36" s="2" t="n">
+        <v>46042</v>
+      </c>
+      <c r="R36" t="n">
+        <v>1</v>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>12317841</v>
+      </c>
+      <c r="B37" t="n">
+        <v>4002310384</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>installation échafaudage sur fuite de ga</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>OR004002310384</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-SECGAZ-0E7315</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>ECHANGEUR GAZ-GAZ FROID E7315 PSIII</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>S-PC-E7315</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>SF1-RPS3</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>BLOQ CLOT CCRP NEFF PART</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>BENMOUSSA1</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="Q37" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="R37" t="n">
+        <v>1</v>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
         </is>
       </c>
     </row>

</xml_diff>